<commit_message>
Implementa la hoja reglas léxicas en el archivo Tokens.xlsx
En esa hoja se realiza un mapeo de los lexemas y su token acompañados de su patrón de escritura para el scanner
</commit_message>
<xml_diff>
--- a/Programa/Tokens.xlsx
+++ b/Programa/Tokens.xlsx
@@ -5,15 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heldy\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heldy\Desktop\PY1_Compi\Programa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E4E727-3250-4179-892A-ED098E4E0CB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2567E55-BC90-46E4-AB5E-5319B8271AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="19935" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="17550" windowHeight="16305" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tokens" sheetId="1" r:id="rId1"/>
+    <sheet name="Reglas léxicas" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="181">
   <si>
     <t>Lexema</t>
   </si>
@@ -406,6 +407,168 @@
   </si>
   <si>
     <t>val booleano</t>
+  </si>
+  <si>
+    <t>Patrón</t>
+  </si>
+  <si>
+    <t>Ejemplo</t>
+  </si>
+  <si>
+    <t>"val"</t>
+  </si>
+  <si>
+    <t>"defun"</t>
+  </si>
+  <si>
+    <t>"int"</t>
+  </si>
+  <si>
+    <t>"float"</t>
+  </si>
+  <si>
+    <t>"bool"</t>
+  </si>
+  <si>
+    <t>"char"</t>
+  </si>
+  <si>
+    <t>"string"</t>
+  </si>
+  <si>
+    <t>"void"</t>
+  </si>
+  <si>
+    <t>"true"</t>
+  </si>
+  <si>
+    <t>"false"</t>
+  </si>
+  <si>
+    <t>"dg"</t>
+  </si>
+  <si>
+    <t>"dl"</t>
+  </si>
+  <si>
+    <t>"if"</t>
+  </si>
+  <si>
+    <t>"elif"</t>
+  </si>
+  <si>
+    <t>"else"</t>
+  </si>
+  <si>
+    <t>"while"</t>
+  </si>
+  <si>
+    <t>"for"</t>
+  </si>
+  <si>
+    <t>"return"</t>
+  </si>
+  <si>
+    <t>"break"</t>
+  </si>
+  <si>
+    <t>"read"</t>
+  </si>
+  <si>
+    <t>"write"</t>
+  </si>
+  <si>
+    <t>"\+"</t>
+  </si>
+  <si>
+    <t>"\-"</t>
+  </si>
+  <si>
+    <t>"\*"</t>
+  </si>
+  <si>
+    <t>"\/"</t>
+  </si>
+  <si>
+    <t>"\//"</t>
+  </si>
+  <si>
+    <t>"mod"</t>
+  </si>
+  <si>
+    <t>"pot"</t>
+  </si>
+  <si>
+    <t>"\&lt;"</t>
+  </si>
+  <si>
+    <t>"\&gt;"</t>
+  </si>
+  <si>
+    <t>"\&lt;="</t>
+  </si>
+  <si>
+    <t>"\&gt;="</t>
+  </si>
+  <si>
+    <t>"\=="</t>
+  </si>
+  <si>
+    <t>"\!="</t>
+  </si>
+  <si>
+    <t>"\λ"</t>
+  </si>
+  <si>
+    <t>"\θ"</t>
+  </si>
+  <si>
+    <t>"\Σ"</t>
+  </si>
+  <si>
+    <t>"¿:"</t>
+  </si>
+  <si>
+    <t>":?"</t>
+  </si>
+  <si>
+    <t>"\є:"</t>
+  </si>
+  <si>
+    <t>":\э"</t>
+  </si>
+  <si>
+    <t>"\ʃ:"</t>
+  </si>
+  <si>
+    <t>":\ʅ"</t>
+  </si>
+  <si>
+    <t>"\»"</t>
+  </si>
+  <si>
+    <t>"\Ͱ"</t>
+  </si>
+  <si>
+    <t>"\,"</t>
+  </si>
+  <si>
+    <t>"\."</t>
+  </si>
+  <si>
+    <t>"|"</t>
+  </si>
+  <si>
+    <t>"¡"</t>
+  </si>
+  <si>
+    <t>"!"</t>
+  </si>
+  <si>
+    <t>0 | [1-9][0-9]*</t>
+  </si>
+  <si>
+    <t>0\.0 | 0\.[0-9][0-9]+[1-9]* | [1-9][0-9]*\.[0-9][1-9]*</t>
   </si>
 </sst>
 </file>
@@ -462,14 +625,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -479,15 +636,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -788,10 +946,10 @@
       <c r="E3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="4"/>
+      <c r="G3" s="6"/>
       <c r="I3" s="2" t="s">
         <v>0</v>
       </c>
@@ -801,10 +959,10 @@
       <c r="K3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="L3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="4"/>
+      <c r="M3" s="6"/>
     </row>
     <row r="4" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C4" s="1" t="s">
@@ -816,10 +974,10 @@
       <c r="E4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="3"/>
+      <c r="F4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="5"/>
       <c r="I4" s="1" t="s">
         <v>76</v>
       </c>
@@ -829,10 +987,10 @@
       <c r="K4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="L4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="3"/>
+      <c r="L4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M4" s="5"/>
     </row>
     <row r="5" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C5" s="1" t="s">
@@ -844,10 +1002,10 @@
       <c r="E5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="3"/>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5"/>
       <c r="I5" s="1" t="s">
         <v>77</v>
       </c>
@@ -857,10 +1015,10 @@
       <c r="K5" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="L5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="3"/>
+      <c r="L5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="5"/>
     </row>
     <row r="6" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C6" s="1" t="s">
@@ -872,10 +1030,10 @@
       <c r="E6" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="3"/>
+      <c r="F6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="5"/>
       <c r="I6" s="1" t="s">
         <v>78</v>
       </c>
@@ -885,10 +1043,10 @@
       <c r="K6" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="L6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" s="3"/>
+      <c r="L6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M6" s="5"/>
     </row>
     <row r="7" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C7" s="1" t="s">
@@ -900,10 +1058,10 @@
       <c r="E7" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="3"/>
+      <c r="F7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="5"/>
       <c r="I7" s="1" t="s">
         <v>79</v>
       </c>
@@ -913,10 +1071,10 @@
       <c r="K7" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M7" s="3"/>
+      <c r="L7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M7" s="5"/>
     </row>
     <row r="8" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C8" s="1" t="s">
@@ -928,10 +1086,10 @@
       <c r="E8" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="3"/>
+      <c r="F8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="5"/>
       <c r="I8" s="1" t="s">
         <v>80</v>
       </c>
@@ -941,10 +1099,10 @@
       <c r="K8" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L8" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M8" s="3"/>
+      <c r="L8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M8" s="5"/>
     </row>
     <row r="9" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
@@ -956,10 +1114,10 @@
       <c r="E9" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="3"/>
+      <c r="F9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="5"/>
       <c r="I9" s="1" t="s">
         <v>81</v>
       </c>
@@ -969,10 +1127,10 @@
       <c r="K9" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M9" s="3"/>
+      <c r="L9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M9" s="5"/>
     </row>
     <row r="10" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C10" s="1" t="s">
@@ -984,10 +1142,10 @@
       <c r="E10" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G10" s="3"/>
+      <c r="F10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="5"/>
       <c r="I10" s="1" t="s">
         <v>82</v>
       </c>
@@ -997,10 +1155,10 @@
       <c r="K10" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M10" s="3"/>
+      <c r="L10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M10" s="5"/>
     </row>
     <row r="11" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C11" s="1" t="s">
@@ -1012,10 +1170,10 @@
       <c r="E11" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G11" s="3"/>
+      <c r="F11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G11" s="5"/>
       <c r="I11" s="1" t="s">
         <v>83</v>
       </c>
@@ -1025,10 +1183,10 @@
       <c r="K11" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M11" s="3"/>
+      <c r="L11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M11" s="5"/>
     </row>
     <row r="12" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C12" s="1" t="s">
@@ -1040,10 +1198,10 @@
       <c r="E12" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G12" s="3"/>
+      <c r="F12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" s="5"/>
       <c r="I12" s="1" t="s">
         <v>84</v>
       </c>
@@ -1053,10 +1211,10 @@
       <c r="K12" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M12" s="3"/>
+      <c r="L12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M12" s="5"/>
     </row>
     <row r="13" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C13" s="1" t="s">
@@ -1068,10 +1226,10 @@
       <c r="E13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G13" s="3"/>
+      <c r="F13" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" s="5"/>
       <c r="I13" s="1" t="s">
         <v>85</v>
       </c>
@@ -1081,10 +1239,10 @@
       <c r="K13" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M13" s="3"/>
+      <c r="L13" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M13" s="5"/>
     </row>
     <row r="14" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C14" s="1" t="s">
@@ -1096,10 +1254,10 @@
       <c r="E14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G14" s="3"/>
+      <c r="F14" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" s="5"/>
       <c r="I14" s="1" t="s">
         <v>86</v>
       </c>
@@ -1109,10 +1267,10 @@
       <c r="K14" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="L14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M14" s="3"/>
+      <c r="L14" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M14" s="5"/>
     </row>
     <row r="15" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C15" s="1" t="s">
@@ -1124,10 +1282,10 @@
       <c r="E15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G15" s="3"/>
+      <c r="F15" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G15" s="5"/>
       <c r="I15" s="1" t="s">
         <v>87</v>
       </c>
@@ -1137,10 +1295,10 @@
       <c r="K15" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M15" s="3"/>
+      <c r="L15" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M15" s="5"/>
     </row>
     <row r="16" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C16" s="1" t="s">
@@ -1152,10 +1310,10 @@
       <c r="E16" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F16" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G16" s="3"/>
+      <c r="F16" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G16" s="5"/>
       <c r="I16" s="1" t="s">
         <v>88</v>
       </c>
@@ -1165,10 +1323,10 @@
       <c r="K16" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L16" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M16" s="3"/>
+      <c r="L16" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M16" s="5"/>
     </row>
     <row r="17" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C17" s="1" t="s">
@@ -1180,10 +1338,10 @@
       <c r="E17" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F17" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G17" s="3"/>
+      <c r="F17" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G17" s="5"/>
       <c r="I17" s="1" t="s">
         <v>89</v>
       </c>
@@ -1193,10 +1351,10 @@
       <c r="K17" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="L17" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M17" s="3"/>
+      <c r="L17" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M17" s="5"/>
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C18" s="1" t="s">
@@ -1208,10 +1366,10 @@
       <c r="E18" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F18" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G18" s="3"/>
+      <c r="F18" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G18" s="5"/>
       <c r="I18" s="1" t="s">
         <v>90</v>
       </c>
@@ -1221,10 +1379,10 @@
       <c r="K18" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="L18" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M18" s="3"/>
+      <c r="L18" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M18" s="5"/>
     </row>
     <row r="19" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C19" s="1" t="s">
@@ -1236,10 +1394,10 @@
       <c r="E19" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F19" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G19" s="3"/>
+      <c r="F19" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G19" s="5"/>
       <c r="I19" s="1" t="s">
         <v>91</v>
       </c>
@@ -1249,10 +1407,10 @@
       <c r="K19" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="L19" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="M19" s="3"/>
+      <c r="L19" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="M19" s="5"/>
     </row>
     <row r="20" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C20" s="1" t="s">
@@ -1264,10 +1422,10 @@
       <c r="E20" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F20" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G20" s="3"/>
+      <c r="F20" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G20" s="5"/>
       <c r="I20" s="1" t="s">
         <v>124</v>
       </c>
@@ -1277,10 +1435,10 @@
       <c r="K20" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L20" s="3" t="s">
+      <c r="L20" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="M20" s="3"/>
+      <c r="M20" s="5"/>
     </row>
     <row r="21" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C21" s="1" t="s">
@@ -1292,10 +1450,10 @@
       <c r="E21" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F21" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G21" s="3"/>
+      <c r="F21" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G21" s="5"/>
       <c r="I21" s="1" t="s">
         <v>125</v>
       </c>
@@ -1305,10 +1463,10 @@
       <c r="K21" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L21" s="3" t="s">
+      <c r="L21" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="M21" s="3"/>
+      <c r="M21" s="5"/>
     </row>
     <row r="22" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C22" s="1" t="s">
@@ -1320,10 +1478,10 @@
       <c r="E22" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F22" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G22" s="3"/>
+      <c r="F22" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G22" s="5"/>
       <c r="I22" s="1" t="s">
         <v>126</v>
       </c>
@@ -1333,10 +1491,10 @@
       <c r="K22" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L22" s="3" t="s">
+      <c r="L22" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="M22" s="3"/>
+      <c r="M22" s="5"/>
     </row>
     <row r="23" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C23" s="1" t="s">
@@ -1348,10 +1506,10 @@
       <c r="E23" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F23" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G23" s="3"/>
+      <c r="F23" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G23" s="5"/>
       <c r="I23" s="1" t="s">
         <v>122</v>
       </c>
@@ -1361,10 +1519,10 @@
       <c r="K23" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L23" s="3" t="s">
+      <c r="L23" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="M23" s="3"/>
+      <c r="M23" s="5"/>
     </row>
     <row r="24" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C24" s="1" t="s">
@@ -1376,10 +1534,10 @@
       <c r="E24" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F24" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G24" s="3"/>
+      <c r="F24" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G24" s="5"/>
       <c r="I24" s="1" t="s">
         <v>119</v>
       </c>
@@ -1389,10 +1547,10 @@
       <c r="K24" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="L24" s="3" t="s">
+      <c r="L24" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="M24" s="3"/>
+      <c r="M24" s="5"/>
     </row>
     <row r="25" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C25" s="1" t="s">
@@ -1404,10 +1562,10 @@
       <c r="E25" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F25" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G25" s="3"/>
+      <c r="F25" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G25" s="5"/>
     </row>
     <row r="26" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C26" s="1" t="s">
@@ -1419,15 +1577,10 @@
       <c r="E26" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F26" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G26" s="3"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
-      <c r="K26" s="6"/>
-      <c r="L26" s="7"/>
-      <c r="M26" s="7"/>
+      <c r="F26" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G26" s="5"/>
     </row>
     <row r="27" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C27" s="1" t="s">
@@ -1439,15 +1592,10 @@
       <c r="E27" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F27" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G27" s="3"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="6"/>
-      <c r="K27" s="6"/>
-      <c r="L27" s="7"/>
-      <c r="M27" s="7"/>
+      <c r="F27" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G27" s="5"/>
     </row>
     <row r="28" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C28" s="1" t="s">
@@ -1459,15 +1607,10 @@
       <c r="E28" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F28" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G28" s="3"/>
-      <c r="I28" s="6"/>
-      <c r="J28" s="6"/>
-      <c r="K28" s="6"/>
-      <c r="L28" s="7"/>
-      <c r="M28" s="7"/>
+      <c r="F28" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G28" s="5"/>
     </row>
     <row r="29" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C29" s="1" t="s">
@@ -1479,10 +1622,10 @@
       <c r="E29" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F29" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G29" s="3"/>
+      <c r="F29" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G29" s="5"/>
     </row>
     <row r="30" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C30" s="1" t="s">
@@ -1494,10 +1637,10 @@
       <c r="E30" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F30" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G30" s="3"/>
+      <c r="F30" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G30" s="5"/>
     </row>
     <row r="31" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C31" s="1" t="s">
@@ -1509,15 +1652,10 @@
       <c r="E31" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F31" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G31" s="3"/>
-      <c r="I31" s="6"/>
-      <c r="J31" s="6"/>
-      <c r="K31" s="6"/>
-      <c r="L31" s="7"/>
-      <c r="M31" s="7"/>
+      <c r="F31" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G31" s="5"/>
     </row>
     <row r="32" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C32" s="1" t="s">
@@ -1529,15 +1667,10 @@
       <c r="E32" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F32" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G32" s="3"/>
-      <c r="I32" s="6"/>
-      <c r="J32" s="6"/>
-      <c r="K32" s="6"/>
-      <c r="L32" s="7"/>
-      <c r="M32" s="7"/>
+      <c r="F32" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G32" s="5"/>
     </row>
     <row r="33" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C33" s="1" t="s">
@@ -1549,15 +1682,10 @@
       <c r="E33" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F33" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G33" s="3"/>
-      <c r="I33" s="6"/>
-      <c r="J33" s="6"/>
-      <c r="K33" s="6"/>
-      <c r="L33" s="7"/>
-      <c r="M33" s="7"/>
+      <c r="F33" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G33" s="5"/>
     </row>
     <row r="34" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C34" s="1" t="s">
@@ -1569,15 +1697,10 @@
       <c r="E34" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F34" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G34" s="3"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="6"/>
-      <c r="K34" s="6"/>
-      <c r="L34" s="7"/>
-      <c r="M34" s="7"/>
+      <c r="F34" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G34" s="5"/>
     </row>
     <row r="35" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C35" s="1" t="s">
@@ -1589,18 +1712,13 @@
       <c r="E35" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F35" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G35" s="3"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="6"/>
-      <c r="K35" s="6"/>
-      <c r="L35" s="7"/>
-      <c r="M35" s="7"/>
+      <c r="F35" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G35" s="5"/>
     </row>
     <row r="36" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="3" t="s">
         <v>65</v>
       </c>
       <c r="D36" s="1" t="s">
@@ -1609,15 +1727,10 @@
       <c r="E36" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F36" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G36" s="3"/>
-      <c r="I36" s="8"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="7"/>
-      <c r="M36" s="7"/>
+      <c r="F36" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G36" s="5"/>
     </row>
     <row r="37" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C37" s="1" t="s">
@@ -1629,70 +1742,18 @@
       <c r="E37" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F37" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G37" s="3"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6"/>
+      <c r="F37" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G37" s="5"/>
+      <c r="I37" s="4"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
       <c r="L37" s="7"/>
       <c r="M37" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="67">
-    <mergeCell ref="L33:M33"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="L35:M35"/>
-    <mergeCell ref="L36:M36"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="L28:M28"/>
-    <mergeCell ref="L31:M31"/>
-    <mergeCell ref="L32:M32"/>
-    <mergeCell ref="L23:M23"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="L27:M27"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="L14:M14"/>
-    <mergeCell ref="L15:M15"/>
-    <mergeCell ref="L16:M16"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="F22:G22"/>
+  <mergeCells count="57">
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="F4:G4"/>
@@ -1708,6 +1769,822 @@
     <mergeCell ref="F14:G14"/>
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="L15:M15"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="L24:M24"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1248E3B3-D830-4831-8AEA-9933D07E9251}">
+  <dimension ref="C5:M39"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="9" max="9" width="12.77734375" customWidth="1"/>
+    <col min="10" max="10" width="45.77734375" customWidth="1"/>
+    <col min="11" max="11" width="15.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="G5" s="6"/>
+      <c r="I5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="M5" s="6"/>
+    </row>
+    <row r="6" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="I6" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+    </row>
+    <row r="7" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="I7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+    </row>
+    <row r="8" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="I8" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+    </row>
+    <row r="9" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="I9" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+    </row>
+    <row r="10" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="I10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+    </row>
+    <row r="11" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="I11" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+    </row>
+    <row r="12" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="I12" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+    </row>
+    <row r="13" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="I13" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+    </row>
+    <row r="14" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="I14" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+    </row>
+    <row r="15" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="I15" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+    </row>
+    <row r="16" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="I16" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+    </row>
+    <row r="17" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="I17" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+    </row>
+    <row r="18" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="I18" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+    </row>
+    <row r="19" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="I19" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+    </row>
+    <row r="20" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C20" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="I20" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+    </row>
+    <row r="21" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C21" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="I21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
+    </row>
+    <row r="22" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C22" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="I22" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
+    </row>
+    <row r="23" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C23" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="I23" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
+    </row>
+    <row r="24" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C24" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="I24" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+    </row>
+    <row r="25" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C25" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="I25" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
+    </row>
+    <row r="26" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C26" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="I26" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="L26" s="5"/>
+      <c r="M26" s="5"/>
+    </row>
+    <row r="27" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C27" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+    </row>
+    <row r="28" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C28" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+    </row>
+    <row r="29" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C29" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+    </row>
+    <row r="30" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C30" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+    </row>
+    <row r="31" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C31" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+    </row>
+    <row r="32" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C32" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+    </row>
+    <row r="33" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C33" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+    </row>
+    <row r="34" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C34" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+    </row>
+    <row r="35" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C35" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+    </row>
+    <row r="36" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C36" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+    </row>
+    <row r="37" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C37" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+    </row>
+    <row r="38" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C38" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+    </row>
+    <row r="39" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="C39" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="4"/>
+      <c r="L39" s="7"/>
+      <c r="M39" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="57">
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="L15:M15"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="L7:M7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Termina la tabla de reglas léxicas
</commit_message>
<xml_diff>
--- a/Programa/Tokens.xlsx
+++ b/Programa/Tokens.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heldy\Desktop\PY1_Compi\Programa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2567E55-BC90-46E4-AB5E-5319B8271AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA750900-E306-45F5-8B55-AEF096817E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="17550" windowHeight="16305" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="19785" windowHeight="16305" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tokens" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="195">
   <si>
     <t>Lexema</t>
   </si>
@@ -565,10 +565,52 @@
     <t>"!"</t>
   </si>
   <si>
-    <t>0 | [1-9][0-9]*</t>
-  </si>
-  <si>
-    <t>0\.0 | 0\.[0-9][0-9]+[1-9]* | [1-9][0-9]*\.[0-9][1-9]*</t>
+    <t>"true" | "false"</t>
+  </si>
+  <si>
+    <t>exponencial</t>
+  </si>
+  <si>
+    <t>LITERAL_EXP</t>
+  </si>
+  <si>
+    <t>(0 |'-? [1-9][0-9]*)[eE](0 | '-?[1-9][0-9]*)</t>
+  </si>
+  <si>
+    <t>(0\.0 | 0\.[0-9]*[1-9] | -?[1-9][0-9]*\.[0-9]*[1-9])</t>
+  </si>
+  <si>
+    <t>(0 | -?[1-9][0-9]*)</t>
+  </si>
+  <si>
+    <t>char literal</t>
+  </si>
+  <si>
+    <t>LITERAL_CHAR</t>
+  </si>
+  <si>
+    <t>Definido con auxiliares de JFLEX</t>
+  </si>
+  <si>
+    <t>0.001239</t>
+  </si>
+  <si>
+    <t>"f"</t>
+  </si>
+  <si>
+    <t>"Hola mundo"</t>
+  </si>
+  <si>
+    <t>"contador"</t>
+  </si>
+  <si>
+    <t>principal</t>
+  </si>
+  <si>
+    <t>PRINCIPAL</t>
+  </si>
+  <si>
+    <t>Char</t>
   </si>
 </sst>
 </file>
@@ -598,7 +640,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -621,11 +663,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -639,13 +707,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -926,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C3:M37"/>
+  <dimension ref="C3:M39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="10.77734375" customWidth="1"/>
@@ -946,10 +1028,10 @@
       <c r="E3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="6"/>
+      <c r="G3" s="5"/>
       <c r="I3" s="2" t="s">
         <v>0</v>
       </c>
@@ -959,10 +1041,10 @@
       <c r="K3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="6" t="s">
+      <c r="L3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="6"/>
+      <c r="M3" s="5"/>
     </row>
     <row r="4" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C4" s="1" t="s">
@@ -974,10 +1056,10 @@
       <c r="E4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="5"/>
+      <c r="F4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="6"/>
       <c r="I4" s="1" t="s">
         <v>76</v>
       </c>
@@ -987,25 +1069,25 @@
       <c r="K4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="L4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="5"/>
+      <c r="L4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M4" s="6"/>
     </row>
     <row r="5" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C5" s="1" t="s">
-        <v>8</v>
+        <v>192</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>9</v>
+        <v>193</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="5"/>
+      <c r="F5" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="9"/>
       <c r="I5" s="1" t="s">
         <v>77</v>
       </c>
@@ -1015,25 +1097,25 @@
       <c r="K5" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="L5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="5"/>
+      <c r="L5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="6"/>
     </row>
     <row r="6" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C6" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="5"/>
+        <v>6</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="6"/>
       <c r="I6" s="1" t="s">
         <v>78</v>
       </c>
@@ -1043,25 +1125,25 @@
       <c r="K6" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="L6" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" s="5"/>
+      <c r="L6" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M6" s="6"/>
     </row>
     <row r="7" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C7" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="5"/>
+      <c r="F7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="6"/>
       <c r="I7" s="1" t="s">
         <v>79</v>
       </c>
@@ -1071,25 +1153,25 @@
       <c r="K7" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L7" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M7" s="5"/>
+      <c r="L7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M7" s="6"/>
     </row>
     <row r="8" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C8" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="5"/>
+      <c r="F8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="6"/>
       <c r="I8" s="1" t="s">
         <v>80</v>
       </c>
@@ -1099,25 +1181,25 @@
       <c r="K8" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L8" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M8" s="5"/>
+      <c r="L8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M8" s="6"/>
     </row>
     <row r="9" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="5"/>
+      <c r="F9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="6"/>
       <c r="I9" s="1" t="s">
         <v>81</v>
       </c>
@@ -1127,25 +1209,25 @@
       <c r="K9" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L9" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M9" s="5"/>
+      <c r="L9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M9" s="6"/>
     </row>
     <row r="10" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C10" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F10" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G10" s="5"/>
+      <c r="F10" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="6"/>
       <c r="I10" s="1" t="s">
         <v>82</v>
       </c>
@@ -1155,25 +1237,25 @@
       <c r="K10" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L10" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M10" s="5"/>
+      <c r="L10" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M10" s="6"/>
     </row>
     <row r="11" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C11" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G11" s="5"/>
+      <c r="F11" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G11" s="6"/>
       <c r="I11" s="1" t="s">
         <v>83</v>
       </c>
@@ -1183,25 +1265,25 @@
       <c r="K11" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L11" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M11" s="5"/>
+      <c r="L11" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M11" s="6"/>
     </row>
     <row r="12" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C12" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G12" s="5"/>
+        <v>108</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" s="6"/>
       <c r="I12" s="1" t="s">
         <v>84</v>
       </c>
@@ -1211,25 +1293,25 @@
       <c r="K12" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L12" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M12" s="5"/>
+      <c r="L12" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M12" s="6"/>
     </row>
     <row r="13" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C13" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F13" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G13" s="5"/>
+      <c r="F13" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" s="6"/>
       <c r="I13" s="1" t="s">
         <v>85</v>
       </c>
@@ -1239,25 +1321,25 @@
       <c r="K13" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L13" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M13" s="5"/>
+      <c r="L13" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M13" s="6"/>
     </row>
     <row r="14" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C14" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G14" s="5"/>
+      <c r="F14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" s="6"/>
       <c r="I14" s="1" t="s">
         <v>86</v>
       </c>
@@ -1267,25 +1349,25 @@
       <c r="K14" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="L14" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M14" s="5"/>
+      <c r="L14" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M14" s="6"/>
     </row>
     <row r="15" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C15" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F15" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G15" s="5"/>
+      <c r="F15" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G15" s="6"/>
       <c r="I15" s="1" t="s">
         <v>87</v>
       </c>
@@ -1295,25 +1377,25 @@
       <c r="K15" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L15" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M15" s="5"/>
+      <c r="L15" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M15" s="6"/>
     </row>
     <row r="16" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C16" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F16" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G16" s="5"/>
+      <c r="F16" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G16" s="6"/>
       <c r="I16" s="1" t="s">
         <v>88</v>
       </c>
@@ -1323,25 +1405,25 @@
       <c r="K16" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L16" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M16" s="5"/>
+      <c r="L16" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M16" s="6"/>
     </row>
     <row r="17" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C17" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F17" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G17" s="5"/>
+      <c r="F17" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G17" s="6"/>
       <c r="I17" s="1" t="s">
         <v>89</v>
       </c>
@@ -1351,25 +1433,25 @@
       <c r="K17" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="L17" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M17" s="5"/>
+      <c r="L17" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M17" s="6"/>
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C18" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F18" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G18" s="5"/>
+      <c r="F18" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G18" s="6"/>
       <c r="I18" s="1" t="s">
         <v>90</v>
       </c>
@@ -1379,25 +1461,25 @@
       <c r="K18" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="L18" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M18" s="5"/>
+      <c r="L18" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M18" s="6"/>
     </row>
     <row r="19" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C19" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F19" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G19" s="5"/>
+      <c r="F19" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G19" s="6"/>
       <c r="I19" s="1" t="s">
         <v>91</v>
       </c>
@@ -1407,25 +1489,25 @@
       <c r="K19" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="L19" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="M19" s="5"/>
+      <c r="L19" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="M19" s="6"/>
     </row>
     <row r="20" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C20" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F20" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G20" s="5"/>
+      <c r="F20" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G20" s="6"/>
       <c r="I20" s="1" t="s">
         <v>124</v>
       </c>
@@ -1435,25 +1517,25 @@
       <c r="K20" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L20" s="5" t="s">
+      <c r="L20" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="M20" s="5"/>
+      <c r="M20" s="6"/>
     </row>
     <row r="21" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C21" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F21" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G21" s="5"/>
+      <c r="F21" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G21" s="6"/>
       <c r="I21" s="1" t="s">
         <v>125</v>
       </c>
@@ -1463,301 +1545,341 @@
       <c r="K21" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L21" s="5" t="s">
+      <c r="L21" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="M21" s="5"/>
+      <c r="M21" s="6"/>
     </row>
     <row r="22" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C22" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F22" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G22" s="5"/>
+      <c r="F22" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G22" s="6"/>
       <c r="I22" s="1" t="s">
-        <v>126</v>
+        <v>180</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>111</v>
+        <v>181</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L22" s="5" t="s">
+      <c r="L22" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="M22" s="5"/>
+      <c r="M22" s="9"/>
     </row>
     <row r="23" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C23" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F23" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G23" s="5"/>
+      <c r="F23" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G23" s="6"/>
       <c r="I23" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K23" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L23" s="5" t="s">
+      <c r="L23" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="M23" s="5"/>
+      <c r="M23" s="6"/>
     </row>
     <row r="24" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C24" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F24" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G24" s="5"/>
+      <c r="F24" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G24" s="6"/>
       <c r="I24" s="1" t="s">
-        <v>119</v>
+        <v>185</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>120</v>
+        <v>186</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="L24" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="L24" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="M24" s="5"/>
+      <c r="M24" s="9"/>
     </row>
     <row r="25" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C25" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G25" s="5"/>
+        <v>6</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G25" s="6"/>
+      <c r="I25" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="M25" s="6"/>
     </row>
     <row r="26" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C26" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F26" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G26" s="5"/>
+      <c r="F26" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G26" s="6"/>
+      <c r="I26" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="L26" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="M26" s="6"/>
     </row>
     <row r="27" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C27" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F27" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G27" s="5"/>
+      <c r="F27" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G27" s="6"/>
     </row>
     <row r="28" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C28" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F28" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G28" s="5"/>
+      <c r="F28" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G28" s="6"/>
     </row>
     <row r="29" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C29" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F29" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G29" s="5"/>
+      <c r="F29" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G29" s="6"/>
     </row>
     <row r="30" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C30" s="1" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F30" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G30" s="5"/>
+      <c r="F30" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G30" s="6"/>
     </row>
     <row r="31" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C31" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F31" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G31" s="5"/>
+      <c r="F31" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G31" s="6"/>
     </row>
     <row r="32" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C32" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G32" s="6"/>
+    </row>
+    <row r="33" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C33" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G32" s="5"/>
-    </row>
-    <row r="33" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C33" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F33" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G33" s="5"/>
-    </row>
-    <row r="34" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F33" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G33" s="6"/>
+    </row>
+    <row r="34" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C34" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F34" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G34" s="5"/>
-    </row>
-    <row r="35" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F34" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G34" s="6"/>
+    </row>
+    <row r="35" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C35" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F35" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G35" s="5"/>
-    </row>
-    <row r="36" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C36" s="3" t="s">
-        <v>65</v>
+      <c r="F35" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G35" s="6"/>
+    </row>
+    <row r="36" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C36" s="1" t="s">
+        <v>64</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F36" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G36" s="5"/>
-    </row>
-    <row r="37" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C37" s="1" t="s">
-        <v>66</v>
+      <c r="F36" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G36" s="6"/>
+    </row>
+    <row r="37" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C37" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F37" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G37" s="5"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="4"/>
-      <c r="K37" s="4"/>
-      <c r="L37" s="7"/>
-      <c r="M37" s="7"/>
+      <c r="F37" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G37" s="6"/>
+    </row>
+    <row r="38" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C38" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G38" s="6"/>
+    </row>
+    <row r="39" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="I39" s="4"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="57">
-    <mergeCell ref="F17:G17"/>
+  <mergeCells count="60">
+    <mergeCell ref="F18:G18"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="F8:G8"/>
@@ -1769,7 +1891,8 @@
     <mergeCell ref="F14:G14"/>
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="F16:G16"/>
-    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F5:G5"/>
     <mergeCell ref="F19:G19"/>
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="F21:G21"/>
@@ -1789,6 +1912,7 @@
     <mergeCell ref="F35:G35"/>
     <mergeCell ref="F36:G36"/>
     <mergeCell ref="F37:G37"/>
+    <mergeCell ref="F38:G38"/>
     <mergeCell ref="L3:M3"/>
     <mergeCell ref="L4:M4"/>
     <mergeCell ref="L5:M5"/>
@@ -1804,12 +1928,14 @@
     <mergeCell ref="L15:M15"/>
     <mergeCell ref="L16:M16"/>
     <mergeCell ref="L17:M17"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="L26:M26"/>
     <mergeCell ref="L18:M18"/>
     <mergeCell ref="L19:M19"/>
     <mergeCell ref="L20:M20"/>
     <mergeCell ref="L21:M21"/>
+    <mergeCell ref="L23:M23"/>
     <mergeCell ref="L22:M22"/>
-    <mergeCell ref="L23:M23"/>
     <mergeCell ref="L24:M24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1818,7 +1944,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1248E3B3-D830-4831-8AEA-9933D07E9251}">
-  <dimension ref="C5:M39"/>
+  <dimension ref="C5:M41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="9" max="9" width="12.77734375" customWidth="1"/>
@@ -1836,10 +1962,10 @@
       <c r="E5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G5" s="6"/>
+      <c r="G5" s="5"/>
       <c r="I5" s="2" t="s">
         <v>0</v>
       </c>
@@ -1849,10 +1975,10 @@
       <c r="K5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="L5" s="6" t="s">
+      <c r="L5" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="M5" s="6"/>
+      <c r="M5" s="5"/>
     </row>
     <row r="6" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C6" s="1" t="s">
@@ -1864,8 +1990,10 @@
       <c r="E6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
+      <c r="F6" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" s="9"/>
       <c r="I6" s="1" t="s">
         <v>76</v>
       </c>
@@ -1875,8 +2003,8 @@
       <c r="K6" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
     </row>
     <row r="7" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C7" s="1" t="s">
@@ -1888,8 +2016,10 @@
       <c r="E7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
+      <c r="F7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="9"/>
       <c r="I7" s="1" t="s">
         <v>77</v>
       </c>
@@ -1899,8 +2029,8 @@
       <c r="K7" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
     </row>
     <row r="8" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C8" s="1" t="s">
@@ -1912,8 +2042,10 @@
       <c r="E8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
+      <c r="F8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="9"/>
       <c r="I8" s="1" t="s">
         <v>78</v>
       </c>
@@ -1923,8 +2055,8 @@
       <c r="K8" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
     </row>
     <row r="9" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
@@ -1936,8 +2068,10 @@
       <c r="E9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
+      <c r="F9" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="G9" s="9"/>
       <c r="I9" s="1" t="s">
         <v>79</v>
       </c>
@@ -1947,8 +2081,8 @@
       <c r="K9" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
     </row>
     <row r="10" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C10" s="1" t="s">
@@ -1960,8 +2094,10 @@
       <c r="E10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
+      <c r="F10" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="9"/>
       <c r="I10" s="1" t="s">
         <v>80</v>
       </c>
@@ -1971,8 +2107,8 @@
       <c r="K10" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
     </row>
     <row r="11" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C11" s="1" t="s">
@@ -1984,8 +2120,10 @@
       <c r="E11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
+      <c r="F11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="9"/>
       <c r="I11" s="1" t="s">
         <v>81</v>
       </c>
@@ -1995,8 +2133,8 @@
       <c r="K11" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
     </row>
     <row r="12" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C12" s="1" t="s">
@@ -2008,8 +2146,10 @@
       <c r="E12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
+      <c r="F12" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="9"/>
       <c r="I12" s="1" t="s">
         <v>82</v>
       </c>
@@ -2019,8 +2159,8 @@
       <c r="K12" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
     </row>
     <row r="13" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C13" s="1" t="s">
@@ -2032,8 +2172,10 @@
       <c r="E13" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
+      <c r="F13" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="9"/>
       <c r="I13" s="1" t="s">
         <v>83</v>
       </c>
@@ -2043,8 +2185,8 @@
       <c r="K13" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
     </row>
     <row r="14" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C14" s="1" t="s">
@@ -2056,8 +2198,10 @@
       <c r="E14" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
+      <c r="F14" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G14" s="9"/>
       <c r="I14" s="1" t="s">
         <v>84</v>
       </c>
@@ -2067,8 +2211,8 @@
       <c r="K14" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
     </row>
     <row r="15" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C15" s="1" t="s">
@@ -2080,8 +2224,10 @@
       <c r="E15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
+      <c r="F15" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G15" s="9"/>
       <c r="I15" s="1" t="s">
         <v>85</v>
       </c>
@@ -2091,8 +2237,8 @@
       <c r="K15" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6"/>
     </row>
     <row r="16" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C16" s="1" t="s">
@@ -2104,8 +2250,10 @@
       <c r="E16" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
+      <c r="F16" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="9"/>
       <c r="I16" s="1" t="s">
         <v>86</v>
       </c>
@@ -2115,8 +2263,8 @@
       <c r="K16" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
+      <c r="L16" s="6"/>
+      <c r="M16" s="6"/>
     </row>
     <row r="17" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C17" s="1" t="s">
@@ -2128,8 +2276,10 @@
       <c r="E17" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
+      <c r="F17" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G17" s="9"/>
       <c r="I17" s="1" t="s">
         <v>87</v>
       </c>
@@ -2139,8 +2289,8 @@
       <c r="K17" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6"/>
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C18" s="1" t="s">
@@ -2152,8 +2302,10 @@
       <c r="E18" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
+      <c r="F18" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G18" s="9"/>
       <c r="I18" s="1" t="s">
         <v>88</v>
       </c>
@@ -2163,8 +2315,8 @@
       <c r="K18" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
+      <c r="L18" s="6"/>
+      <c r="M18" s="6"/>
     </row>
     <row r="19" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C19" s="1" t="s">
@@ -2176,8 +2328,10 @@
       <c r="E19" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
+      <c r="F19" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="G19" s="9"/>
       <c r="I19" s="1" t="s">
         <v>89</v>
       </c>
@@ -2187,8 +2341,8 @@
       <c r="K19" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6"/>
     </row>
     <row r="20" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C20" s="1" t="s">
@@ -2200,8 +2354,10 @@
       <c r="E20" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
+      <c r="F20" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G20" s="9"/>
       <c r="I20" s="1" t="s">
         <v>90</v>
       </c>
@@ -2211,8 +2367,8 @@
       <c r="K20" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
+      <c r="L20" s="6"/>
+      <c r="M20" s="6"/>
     </row>
     <row r="21" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C21" s="1" t="s">
@@ -2224,8 +2380,10 @@
       <c r="E21" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
+      <c r="F21" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G21" s="9"/>
       <c r="I21" s="1" t="s">
         <v>91</v>
       </c>
@@ -2235,8 +2393,8 @@
       <c r="K21" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
+      <c r="L21" s="6"/>
+      <c r="M21" s="6"/>
     </row>
     <row r="22" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C22" s="1" t="s">
@@ -2248,19 +2406,23 @@
       <c r="E22" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
+      <c r="F22" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G22" s="9"/>
       <c r="I22" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="J22" s="1" t="s">
-        <v>179</v>
+      <c r="J22" s="3" t="s">
+        <v>184</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
+      <c r="L22" s="6">
+        <v>124210</v>
+      </c>
+      <c r="M22" s="6"/>
     </row>
     <row r="23" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C23" s="1" t="s">
@@ -2272,19 +2434,23 @@
       <c r="E23" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
+      <c r="F23" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G23" s="9"/>
       <c r="I23" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="J23" s="1" t="s">
-        <v>180</v>
+      <c r="J23" s="3" t="s">
+        <v>183</v>
       </c>
       <c r="K23" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
+      <c r="L23" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="M23" s="6"/>
     </row>
     <row r="24" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C24" s="1" t="s">
@@ -2296,17 +2462,23 @@
       <c r="E24" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
+      <c r="F24" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G24" s="9"/>
       <c r="I24" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="J24" s="1"/>
+        <v>180</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>182</v>
+      </c>
       <c r="K24" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
+        <v>181</v>
+      </c>
+      <c r="L24" s="7">
+        <v>40000000000</v>
+      </c>
+      <c r="M24" s="6"/>
     </row>
     <row r="25" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C25" s="1" t="s">
@@ -2318,17 +2490,23 @@
       <c r="E25" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
+      <c r="F25" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="G25" s="9"/>
       <c r="I25" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="J25" s="1"/>
+        <v>126</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>179</v>
+      </c>
       <c r="K25" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
+        <v>111</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M25" s="6"/>
     </row>
     <row r="26" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C26" s="1" t="s">
@@ -2340,17 +2518,23 @@
       <c r="E26" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
+      <c r="F26" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="G26" s="9"/>
       <c r="I26" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="J26" s="1"/>
+        <v>185</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>187</v>
+      </c>
       <c r="K26" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="L26" s="5"/>
-      <c r="M26" s="5"/>
+        <v>186</v>
+      </c>
+      <c r="L26" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="M26" s="9"/>
     </row>
     <row r="27" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C27" s="1" t="s">
@@ -2362,8 +2546,23 @@
       <c r="E27" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
+      <c r="F27" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G27" s="9"/>
+      <c r="I27" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L27" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="M27" s="6"/>
     </row>
     <row r="28" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C28" s="1" t="s">
@@ -2375,8 +2574,23 @@
       <c r="E28" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
+      <c r="F28" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G28" s="9"/>
+      <c r="I28" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="M28" s="6"/>
     </row>
     <row r="29" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C29" s="1" t="s">
@@ -2388,8 +2602,10 @@
       <c r="E29" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
+      <c r="F29" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G29" s="9"/>
     </row>
     <row r="30" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C30" s="1" t="s">
@@ -2401,8 +2617,10 @@
       <c r="E30" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
+      <c r="F30" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G30" s="9"/>
     </row>
     <row r="31" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C31" s="1" t="s">
@@ -2414,8 +2632,10 @@
       <c r="E31" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
+      <c r="F31" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G31" s="9"/>
     </row>
     <row r="32" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C32" s="1" t="s">
@@ -2427,10 +2647,12 @@
       <c r="E32" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
-    </row>
-    <row r="33" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F32" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="G32" s="9"/>
+    </row>
+    <row r="33" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C33" s="1" t="s">
         <v>60</v>
       </c>
@@ -2440,10 +2662,12 @@
       <c r="E33" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-    </row>
-    <row r="34" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F33" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G33" s="9"/>
+    </row>
+    <row r="34" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C34" s="1" t="s">
         <v>61</v>
       </c>
@@ -2453,10 +2677,12 @@
       <c r="E34" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
-    </row>
-    <row r="35" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F34" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="G34" s="9"/>
+    </row>
+    <row r="35" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C35" s="1" t="s">
         <v>62</v>
       </c>
@@ -2466,10 +2692,12 @@
       <c r="E35" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-    </row>
-    <row r="36" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F35" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="G35" s="9"/>
+    </row>
+    <row r="36" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C36" s="1" t="s">
         <v>63</v>
       </c>
@@ -2479,10 +2707,12 @@
       <c r="E36" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-    </row>
-    <row r="37" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F36" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="G36" s="9"/>
+    </row>
+    <row r="37" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C37" s="1" t="s">
         <v>64</v>
       </c>
@@ -2492,10 +2722,12 @@
       <c r="E37" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
-    </row>
-    <row r="38" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F37" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="G37" s="9"/>
+    </row>
+    <row r="38" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C38" s="3" t="s">
         <v>65</v>
       </c>
@@ -2505,10 +2737,12 @@
       <c r="E38" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F38" s="5"/>
-      <c r="G38" s="5"/>
-    </row>
-    <row r="39" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F38" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="G38" s="11"/>
+    </row>
+    <row r="39" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C39" s="1" t="s">
         <v>66</v>
       </c>
@@ -2518,37 +2752,41 @@
       <c r="E39" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F39" s="5"/>
-      <c r="G39" s="5"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="4"/>
-      <c r="K39" s="4"/>
-      <c r="L39" s="7"/>
-      <c r="M39" s="7"/>
+      <c r="F39" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G39" s="9"/>
+    </row>
+    <row r="41" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="I41" s="4"/>
+      <c r="J41" s="4"/>
+      <c r="K41" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="57">
-    <mergeCell ref="F37:G37"/>
+  <mergeCells count="59">
     <mergeCell ref="F38:G38"/>
     <mergeCell ref="F39:G39"/>
     <mergeCell ref="F31:G31"/>
     <mergeCell ref="F32:G32"/>
     <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F34:G34"/>
     <mergeCell ref="F35:G35"/>
     <mergeCell ref="F36:G36"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="F34:G34"/>
     <mergeCell ref="F30:G30"/>
     <mergeCell ref="F23:G23"/>
     <mergeCell ref="L23:M23"/>
     <mergeCell ref="F24:G24"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="L27:M27"/>
     <mergeCell ref="L24:M24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F29:G29"/>
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="L20:M20"/>
     <mergeCell ref="F21:G21"/>

</xml_diff>

<commit_message>
Define macros, símbolos y palabras reservadas
</commit_message>
<xml_diff>
--- a/Programa/Tokens.xlsx
+++ b/Programa/Tokens.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heldy\Desktop\PY1_Compi\Programa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA750900-E306-45F5-8B55-AEF096817E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9755EF33-8206-47BB-9FBA-5C2949660F4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="19785" windowHeight="16305" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33180" yWindow="3615" windowWidth="17280" windowHeight="9420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tokens" sheetId="1" r:id="rId1"/>
@@ -577,9 +577,6 @@
     <t>(0 |'-? [1-9][0-9]*)[eE](0 | '-?[1-9][0-9]*)</t>
   </si>
   <si>
-    <t>(0\.0 | 0\.[0-9]*[1-9] | -?[1-9][0-9]*\.[0-9]*[1-9])</t>
-  </si>
-  <si>
     <t>(0 | -?[1-9][0-9]*)</t>
   </si>
   <si>
@@ -611,6 +608,9 @@
   </si>
   <si>
     <t>Char</t>
+  </si>
+  <si>
+    <t>(0\.0 | 0\.[0-9]*[1-9] | [1-9][0-9]*\.[0-9]*[1-9])</t>
   </si>
 </sst>
 </file>
@@ -707,7 +707,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -716,16 +725,7 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1028,10 +1028,10 @@
       <c r="E3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="5"/>
+      <c r="G3" s="11"/>
       <c r="I3" s="2" t="s">
         <v>0</v>
       </c>
@@ -1041,10 +1041,10 @@
       <c r="K3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="L3" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="5"/>
+      <c r="M3" s="11"/>
     </row>
     <row r="4" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C4" s="1" t="s">
@@ -1056,10 +1056,10 @@
       <c r="E4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="6"/>
+      <c r="F4" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="9"/>
       <c r="I4" s="1" t="s">
         <v>76</v>
       </c>
@@ -1069,25 +1069,25 @@
       <c r="K4" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="L4" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M4" s="6"/>
+      <c r="L4" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M4" s="9"/>
     </row>
     <row r="5" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C5" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>192</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>193</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="9"/>
+      <c r="F5" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="8"/>
       <c r="I5" s="1" t="s">
         <v>77</v>
       </c>
@@ -1097,10 +1097,10 @@
       <c r="K5" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="L5" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M5" s="6"/>
+      <c r="L5" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C6" s="1" t="s">
@@ -1112,10 +1112,10 @@
       <c r="E6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="6"/>
+      <c r="F6" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="9"/>
       <c r="I6" s="1" t="s">
         <v>78</v>
       </c>
@@ -1125,10 +1125,10 @@
       <c r="K6" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="L6" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M6" s="6"/>
+      <c r="L6" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M6" s="9"/>
     </row>
     <row r="7" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C7" s="1" t="s">
@@ -1140,10 +1140,10 @@
       <c r="E7" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="6"/>
+      <c r="F7" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="9"/>
       <c r="I7" s="1" t="s">
         <v>79</v>
       </c>
@@ -1153,10 +1153,10 @@
       <c r="K7" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L7" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M7" s="6"/>
+      <c r="L7" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M7" s="9"/>
     </row>
     <row r="8" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C8" s="1" t="s">
@@ -1168,10 +1168,10 @@
       <c r="E8" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="6"/>
+      <c r="F8" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="9"/>
       <c r="I8" s="1" t="s">
         <v>80</v>
       </c>
@@ -1181,10 +1181,10 @@
       <c r="K8" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L8" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M8" s="6"/>
+      <c r="L8" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M8" s="9"/>
     </row>
     <row r="9" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
@@ -1196,10 +1196,10 @@
       <c r="E9" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="6"/>
+      <c r="F9" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="9"/>
       <c r="I9" s="1" t="s">
         <v>81</v>
       </c>
@@ -1209,10 +1209,10 @@
       <c r="K9" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L9" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M9" s="6"/>
+      <c r="L9" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M9" s="9"/>
     </row>
     <row r="10" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C10" s="1" t="s">
@@ -1224,10 +1224,10 @@
       <c r="E10" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F10" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G10" s="6"/>
+      <c r="F10" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="9"/>
       <c r="I10" s="1" t="s">
         <v>82</v>
       </c>
@@ -1237,10 +1237,10 @@
       <c r="K10" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L10" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M10" s="6"/>
+      <c r="L10" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M10" s="9"/>
     </row>
     <row r="11" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C11" s="1" t="s">
@@ -1252,10 +1252,10 @@
       <c r="E11" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F11" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G11" s="6"/>
+      <c r="F11" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G11" s="9"/>
       <c r="I11" s="1" t="s">
         <v>83</v>
       </c>
@@ -1265,10 +1265,10 @@
       <c r="K11" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L11" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M11" s="6"/>
+      <c r="L11" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M11" s="9"/>
     </row>
     <row r="12" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C12" s="1" t="s">
@@ -1280,10 +1280,10 @@
       <c r="E12" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F12" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G12" s="6"/>
+      <c r="F12" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" s="9"/>
       <c r="I12" s="1" t="s">
         <v>84</v>
       </c>
@@ -1293,10 +1293,10 @@
       <c r="K12" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L12" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M12" s="6"/>
+      <c r="L12" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M12" s="9"/>
     </row>
     <row r="13" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C13" s="1" t="s">
@@ -1308,10 +1308,10 @@
       <c r="E13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G13" s="6"/>
+      <c r="F13" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" s="9"/>
       <c r="I13" s="1" t="s">
         <v>85</v>
       </c>
@@ -1321,10 +1321,10 @@
       <c r="K13" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L13" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M13" s="6"/>
+      <c r="L13" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M13" s="9"/>
     </row>
     <row r="14" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C14" s="1" t="s">
@@ -1336,10 +1336,10 @@
       <c r="E14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G14" s="6"/>
+      <c r="F14" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" s="9"/>
       <c r="I14" s="1" t="s">
         <v>86</v>
       </c>
@@ -1349,10 +1349,10 @@
       <c r="K14" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="L14" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M14" s="6"/>
+      <c r="L14" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M14" s="9"/>
     </row>
     <row r="15" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C15" s="1" t="s">
@@ -1364,10 +1364,10 @@
       <c r="E15" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G15" s="6"/>
+      <c r="F15" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G15" s="9"/>
       <c r="I15" s="1" t="s">
         <v>87</v>
       </c>
@@ -1377,10 +1377,10 @@
       <c r="K15" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="L15" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M15" s="6"/>
+      <c r="L15" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M15" s="9"/>
     </row>
     <row r="16" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C16" s="1" t="s">
@@ -1392,10 +1392,10 @@
       <c r="E16" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F16" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G16" s="6"/>
+      <c r="F16" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G16" s="9"/>
       <c r="I16" s="1" t="s">
         <v>88</v>
       </c>
@@ -1405,10 +1405,10 @@
       <c r="K16" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="L16" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M16" s="6"/>
+      <c r="L16" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M16" s="9"/>
     </row>
     <row r="17" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C17" s="1" t="s">
@@ -1420,10 +1420,10 @@
       <c r="E17" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F17" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G17" s="6"/>
+      <c r="F17" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G17" s="9"/>
       <c r="I17" s="1" t="s">
         <v>89</v>
       </c>
@@ -1433,10 +1433,10 @@
       <c r="K17" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="L17" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M17" s="6"/>
+      <c r="L17" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M17" s="9"/>
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C18" s="1" t="s">
@@ -1448,10 +1448,10 @@
       <c r="E18" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G18" s="6"/>
+      <c r="F18" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G18" s="9"/>
       <c r="I18" s="1" t="s">
         <v>90</v>
       </c>
@@ -1461,10 +1461,10 @@
       <c r="K18" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="L18" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M18" s="6"/>
+      <c r="L18" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M18" s="9"/>
     </row>
     <row r="19" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C19" s="1" t="s">
@@ -1476,10 +1476,10 @@
       <c r="E19" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F19" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G19" s="6"/>
+      <c r="F19" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G19" s="9"/>
       <c r="I19" s="1" t="s">
         <v>91</v>
       </c>
@@ -1489,10 +1489,10 @@
       <c r="K19" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="L19" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="M19" s="6"/>
+      <c r="L19" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="M19" s="9"/>
     </row>
     <row r="20" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C20" s="1" t="s">
@@ -1504,10 +1504,10 @@
       <c r="E20" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F20" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G20" s="6"/>
+      <c r="F20" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G20" s="9"/>
       <c r="I20" s="1" t="s">
         <v>124</v>
       </c>
@@ -1517,10 +1517,10 @@
       <c r="K20" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L20" s="6" t="s">
+      <c r="L20" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="M20" s="6"/>
+      <c r="M20" s="9"/>
     </row>
     <row r="21" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C21" s="1" t="s">
@@ -1532,10 +1532,10 @@
       <c r="E21" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F21" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G21" s="6"/>
+      <c r="F21" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G21" s="9"/>
       <c r="I21" s="1" t="s">
         <v>125</v>
       </c>
@@ -1545,10 +1545,10 @@
       <c r="K21" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L21" s="6" t="s">
+      <c r="L21" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="M21" s="6"/>
+      <c r="M21" s="9"/>
     </row>
     <row r="22" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C22" s="1" t="s">
@@ -1560,10 +1560,10 @@
       <c r="E22" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G22" s="6"/>
+      <c r="F22" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G22" s="9"/>
       <c r="I22" s="1" t="s">
         <v>180</v>
       </c>
@@ -1573,10 +1573,10 @@
       <c r="K22" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L22" s="8" t="s">
+      <c r="L22" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="M22" s="9"/>
+      <c r="M22" s="8"/>
     </row>
     <row r="23" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C23" s="1" t="s">
@@ -1588,10 +1588,10 @@
       <c r="E23" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F23" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G23" s="6"/>
+      <c r="F23" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G23" s="9"/>
       <c r="I23" s="1" t="s">
         <v>126</v>
       </c>
@@ -1601,10 +1601,10 @@
       <c r="K23" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L23" s="6" t="s">
+      <c r="L23" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="M23" s="6"/>
+      <c r="M23" s="9"/>
     </row>
     <row r="24" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C24" s="1" t="s">
@@ -1616,23 +1616,23 @@
       <c r="E24" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G24" s="6"/>
+      <c r="F24" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G24" s="9"/>
       <c r="I24" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="J24" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>186</v>
       </c>
       <c r="K24" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L24" s="8" t="s">
+      <c r="L24" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="M24" s="9"/>
+      <c r="M24" s="8"/>
     </row>
     <row r="25" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C25" s="1" t="s">
@@ -1644,10 +1644,10 @@
       <c r="E25" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F25" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G25" s="6"/>
+      <c r="F25" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G25" s="9"/>
       <c r="I25" s="1" t="s">
         <v>122</v>
       </c>
@@ -1657,10 +1657,10 @@
       <c r="K25" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L25" s="6" t="s">
+      <c r="L25" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="M25" s="6"/>
+      <c r="M25" s="9"/>
     </row>
     <row r="26" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C26" s="1" t="s">
@@ -1672,10 +1672,10 @@
       <c r="E26" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G26" s="6"/>
+      <c r="F26" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G26" s="9"/>
       <c r="I26" s="1" t="s">
         <v>119</v>
       </c>
@@ -1685,10 +1685,10 @@
       <c r="K26" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="L26" s="6" t="s">
+      <c r="L26" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="M26" s="6"/>
+      <c r="M26" s="9"/>
     </row>
     <row r="27" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C27" s="1" t="s">
@@ -1700,10 +1700,10 @@
       <c r="E27" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F27" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G27" s="6"/>
+      <c r="F27" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G27" s="9"/>
     </row>
     <row r="28" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C28" s="1" t="s">
@@ -1715,10 +1715,10 @@
       <c r="E28" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F28" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G28" s="6"/>
+      <c r="F28" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G28" s="9"/>
     </row>
     <row r="29" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C29" s="1" t="s">
@@ -1730,10 +1730,10 @@
       <c r="E29" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F29" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G29" s="6"/>
+      <c r="F29" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G29" s="9"/>
     </row>
     <row r="30" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C30" s="1" t="s">
@@ -1745,10 +1745,10 @@
       <c r="E30" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F30" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G30" s="6"/>
+      <c r="F30" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G30" s="9"/>
     </row>
     <row r="31" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C31" s="1" t="s">
@@ -1760,10 +1760,10 @@
       <c r="E31" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F31" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G31" s="6"/>
+      <c r="F31" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G31" s="9"/>
     </row>
     <row r="32" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C32" s="1" t="s">
@@ -1775,10 +1775,10 @@
       <c r="E32" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F32" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G32" s="6"/>
+      <c r="F32" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G32" s="9"/>
     </row>
     <row r="33" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C33" s="1" t="s">
@@ -1790,10 +1790,10 @@
       <c r="E33" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F33" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G33" s="6"/>
+      <c r="F33" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G33" s="9"/>
     </row>
     <row r="34" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C34" s="1" t="s">
@@ -1805,10 +1805,10 @@
       <c r="E34" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F34" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G34" s="6"/>
+      <c r="F34" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G34" s="9"/>
     </row>
     <row r="35" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C35" s="1" t="s">
@@ -1820,10 +1820,10 @@
       <c r="E35" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F35" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G35" s="6"/>
+      <c r="F35" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G35" s="9"/>
     </row>
     <row r="36" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C36" s="1" t="s">
@@ -1835,10 +1835,10 @@
       <c r="E36" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F36" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G36" s="6"/>
+      <c r="F36" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G36" s="9"/>
     </row>
     <row r="37" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C37" s="3" t="s">
@@ -1850,10 +1850,10 @@
       <c r="E37" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F37" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G37" s="6"/>
+      <c r="F37" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G37" s="9"/>
     </row>
     <row r="38" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C38" s="1" t="s">
@@ -1865,10 +1865,10 @@
       <c r="E38" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="F38" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G38" s="6"/>
+      <c r="F38" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G38" s="9"/>
     </row>
     <row r="39" spans="3:11" x14ac:dyDescent="0.3">
       <c r="I39" s="4"/>
@@ -1877,6 +1877,50 @@
     </row>
   </sheetData>
   <mergeCells count="60">
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="L15:M15"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F23:G23"/>
     <mergeCell ref="F18:G18"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="F4:G4"/>
@@ -1893,50 +1937,6 @@
     <mergeCell ref="F16:G16"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="F5:G5"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="L7:M7"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="L14:M14"/>
-    <mergeCell ref="L15:M15"/>
-    <mergeCell ref="L16:M16"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="L25:M25"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="L23:M23"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="L24:M24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1962,10 +1962,10 @@
       <c r="E5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="G5" s="5"/>
+      <c r="G5" s="11"/>
       <c r="I5" s="2" t="s">
         <v>0</v>
       </c>
@@ -1975,10 +1975,10 @@
       <c r="K5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="L5" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="M5" s="5"/>
+      <c r="M5" s="11"/>
     </row>
     <row r="6" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C6" s="1" t="s">
@@ -1990,10 +1990,10 @@
       <c r="E6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="9"/>
+      <c r="G6" s="8"/>
       <c r="I6" s="1" t="s">
         <v>76</v>
       </c>
@@ -2003,8 +2003,8 @@
       <c r="K6" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
     </row>
     <row r="7" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C7" s="1" t="s">
@@ -2016,10 +2016,10 @@
       <c r="E7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="9"/>
+      <c r="G7" s="8"/>
       <c r="I7" s="1" t="s">
         <v>77</v>
       </c>
@@ -2029,8 +2029,8 @@
       <c r="K7" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
     </row>
     <row r="8" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C8" s="1" t="s">
@@ -2042,10 +2042,10 @@
       <c r="E8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="9"/>
+      <c r="G8" s="8"/>
       <c r="I8" s="1" t="s">
         <v>78</v>
       </c>
@@ -2055,8 +2055,8 @@
       <c r="K8" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
     </row>
     <row r="9" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
@@ -2068,10 +2068,10 @@
       <c r="E9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>194</v>
-      </c>
-      <c r="G9" s="9"/>
+      <c r="F9" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="G9" s="8"/>
       <c r="I9" s="1" t="s">
         <v>79</v>
       </c>
@@ -2081,8 +2081,8 @@
       <c r="K9" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
     </row>
     <row r="10" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C10" s="1" t="s">
@@ -2094,10 +2094,10 @@
       <c r="E10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="9"/>
+      <c r="G10" s="8"/>
       <c r="I10" s="1" t="s">
         <v>80</v>
       </c>
@@ -2107,8 +2107,8 @@
       <c r="K10" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
     </row>
     <row r="11" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C11" s="1" t="s">
@@ -2120,10 +2120,10 @@
       <c r="E11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G11" s="9"/>
+      <c r="G11" s="8"/>
       <c r="I11" s="1" t="s">
         <v>81</v>
       </c>
@@ -2133,8 +2133,8 @@
       <c r="K11" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
     </row>
     <row r="12" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C12" s="1" t="s">
@@ -2146,10 +2146,10 @@
       <c r="E12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="G12" s="9"/>
+      <c r="G12" s="8"/>
       <c r="I12" s="1" t="s">
         <v>82</v>
       </c>
@@ -2159,8 +2159,8 @@
       <c r="K12" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
     </row>
     <row r="13" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C13" s="1" t="s">
@@ -2172,10 +2172,10 @@
       <c r="E13" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G13" s="9"/>
+      <c r="G13" s="8"/>
       <c r="I13" s="1" t="s">
         <v>83</v>
       </c>
@@ -2185,8 +2185,8 @@
       <c r="K13" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
     </row>
     <row r="14" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C14" s="1" t="s">
@@ -2198,10 +2198,10 @@
       <c r="E14" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="G14" s="9"/>
+      <c r="G14" s="8"/>
       <c r="I14" s="1" t="s">
         <v>84</v>
       </c>
@@ -2211,8 +2211,8 @@
       <c r="K14" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
     </row>
     <row r="15" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C15" s="1" t="s">
@@ -2224,10 +2224,10 @@
       <c r="E15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="G15" s="9"/>
+      <c r="G15" s="8"/>
       <c r="I15" s="1" t="s">
         <v>85</v>
       </c>
@@ -2237,8 +2237,8 @@
       <c r="K15" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
     </row>
     <row r="16" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C16" s="1" t="s">
@@ -2250,10 +2250,10 @@
       <c r="E16" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="9"/>
+      <c r="G16" s="8"/>
       <c r="I16" s="1" t="s">
         <v>86</v>
       </c>
@@ -2263,8 +2263,8 @@
       <c r="K16" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="L16" s="6"/>
-      <c r="M16" s="6"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
     </row>
     <row r="17" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C17" s="1" t="s">
@@ -2276,10 +2276,10 @@
       <c r="E17" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G17" s="9"/>
+      <c r="G17" s="8"/>
       <c r="I17" s="1" t="s">
         <v>87</v>
       </c>
@@ -2289,8 +2289,8 @@
       <c r="K17" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="L17" s="6"/>
-      <c r="M17" s="6"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C18" s="1" t="s">
@@ -2302,10 +2302,10 @@
       <c r="E18" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="G18" s="9"/>
+      <c r="G18" s="8"/>
       <c r="I18" s="1" t="s">
         <v>88</v>
       </c>
@@ -2315,8 +2315,8 @@
       <c r="K18" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
     </row>
     <row r="19" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C19" s="1" t="s">
@@ -2328,10 +2328,10 @@
       <c r="E19" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="G19" s="9"/>
+      <c r="G19" s="8"/>
       <c r="I19" s="1" t="s">
         <v>89</v>
       </c>
@@ -2341,8 +2341,8 @@
       <c r="K19" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="L19" s="6"/>
-      <c r="M19" s="6"/>
+      <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
     </row>
     <row r="20" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C20" s="1" t="s">
@@ -2354,10 +2354,10 @@
       <c r="E20" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="G20" s="9"/>
+      <c r="G20" s="8"/>
       <c r="I20" s="1" t="s">
         <v>90</v>
       </c>
@@ -2367,8 +2367,8 @@
       <c r="K20" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="L20" s="6"/>
-      <c r="M20" s="6"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
     </row>
     <row r="21" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C21" s="1" t="s">
@@ -2380,10 +2380,10 @@
       <c r="E21" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G21" s="9"/>
+      <c r="G21" s="8"/>
       <c r="I21" s="1" t="s">
         <v>91</v>
       </c>
@@ -2393,8 +2393,8 @@
       <c r="K21" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="L21" s="6"/>
-      <c r="M21" s="6"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
     </row>
     <row r="22" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C22" s="1" t="s">
@@ -2406,23 +2406,23 @@
       <c r="E22" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="G22" s="9"/>
+      <c r="G22" s="8"/>
       <c r="I22" s="1" t="s">
         <v>124</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="L22" s="6">
+      <c r="L22" s="9">
         <v>124210</v>
       </c>
-      <c r="M22" s="6"/>
+      <c r="M22" s="9"/>
     </row>
     <row r="23" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C23" s="1" t="s">
@@ -2434,23 +2434,23 @@
       <c r="E23" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="F23" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G23" s="9"/>
+      <c r="G23" s="8"/>
       <c r="I23" s="1" t="s">
         <v>125</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="K23" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="L23" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="M23" s="6"/>
+      <c r="L23" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="M23" s="9"/>
     </row>
     <row r="24" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C24" s="1" t="s">
@@ -2462,10 +2462,10 @@
       <c r="E24" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G24" s="9"/>
+      <c r="G24" s="8"/>
       <c r="I24" s="1" t="s">
         <v>180</v>
       </c>
@@ -2475,10 +2475,10 @@
       <c r="K24" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="L24" s="7">
+      <c r="L24" s="10">
         <v>40000000000</v>
       </c>
-      <c r="M24" s="6"/>
+      <c r="M24" s="9"/>
     </row>
     <row r="25" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C25" s="1" t="s">
@@ -2490,10 +2490,10 @@
       <c r="E25" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G25" s="9"/>
+      <c r="G25" s="8"/>
       <c r="I25" s="1" t="s">
         <v>126</v>
       </c>
@@ -2503,10 +2503,10 @@
       <c r="K25" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="L25" s="6" t="s">
+      <c r="L25" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="M25" s="6"/>
+      <c r="M25" s="9"/>
     </row>
     <row r="26" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C26" s="1" t="s">
@@ -2518,23 +2518,23 @@
       <c r="E26" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F26" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="G26" s="9"/>
+      <c r="G26" s="8"/>
       <c r="I26" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="K26" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="J26" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="K26" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="L26" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="M26" s="9"/>
+      <c r="L26" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="M26" s="8"/>
     </row>
     <row r="27" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C27" s="1" t="s">
@@ -2546,23 +2546,23 @@
       <c r="E27" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G27" s="9"/>
+      <c r="G27" s="8"/>
       <c r="I27" s="1" t="s">
         <v>122</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K27" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="L27" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="M27" s="6"/>
+      <c r="L27" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="M27" s="9"/>
     </row>
     <row r="28" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C28" s="1" t="s">
@@ -2574,23 +2574,23 @@
       <c r="E28" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="F28" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="G28" s="9"/>
+      <c r="G28" s="8"/>
       <c r="I28" s="1" t="s">
         <v>119</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K28" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="L28" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="M28" s="6"/>
+      <c r="L28" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="M28" s="9"/>
     </row>
     <row r="29" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C29" s="1" t="s">
@@ -2602,10 +2602,10 @@
       <c r="E29" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F29" s="8" t="s">
+      <c r="F29" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G29" s="9"/>
+      <c r="G29" s="8"/>
     </row>
     <row r="30" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C30" s="1" t="s">
@@ -2617,10 +2617,10 @@
       <c r="E30" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="F30" s="8" t="s">
+      <c r="F30" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G30" s="9"/>
+      <c r="G30" s="8"/>
     </row>
     <row r="31" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C31" s="1" t="s">
@@ -2632,10 +2632,10 @@
       <c r="E31" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="F31" s="8" t="s">
+      <c r="F31" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G31" s="9"/>
+      <c r="G31" s="8"/>
     </row>
     <row r="32" spans="3:13" x14ac:dyDescent="0.3">
       <c r="C32" s="1" t="s">
@@ -2647,10 +2647,10 @@
       <c r="E32" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F32" s="8" t="s">
+      <c r="F32" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="G32" s="9"/>
+      <c r="G32" s="8"/>
     </row>
     <row r="33" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C33" s="1" t="s">
@@ -2662,10 +2662,10 @@
       <c r="E33" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F33" s="8" t="s">
+      <c r="F33" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G33" s="9"/>
+      <c r="G33" s="8"/>
     </row>
     <row r="34" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C34" s="1" t="s">
@@ -2677,10 +2677,10 @@
       <c r="E34" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F34" s="8" t="s">
+      <c r="F34" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="G34" s="9"/>
+      <c r="G34" s="8"/>
     </row>
     <row r="35" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C35" s="1" t="s">
@@ -2692,10 +2692,10 @@
       <c r="E35" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="F35" s="8" t="s">
+      <c r="F35" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G35" s="9"/>
+      <c r="G35" s="8"/>
     </row>
     <row r="36" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C36" s="1" t="s">
@@ -2707,10 +2707,10 @@
       <c r="E36" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F36" s="8" t="s">
+      <c r="F36" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="G36" s="9"/>
+      <c r="G36" s="8"/>
     </row>
     <row r="37" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C37" s="1" t="s">
@@ -2722,10 +2722,10 @@
       <c r="E37" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="F37" s="8" t="s">
+      <c r="F37" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="G37" s="9"/>
+      <c r="G37" s="8"/>
     </row>
     <row r="38" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C38" s="3" t="s">
@@ -2737,10 +2737,10 @@
       <c r="E38" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="F38" s="10" t="s">
+      <c r="F38" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="G38" s="11"/>
+      <c r="G38" s="6"/>
     </row>
     <row r="39" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C39" s="1" t="s">
@@ -2752,10 +2752,10 @@
       <c r="E39" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F39" s="8" t="s">
+      <c r="F39" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="G39" s="9"/>
+      <c r="G39" s="8"/>
     </row>
     <row r="41" spans="3:11" x14ac:dyDescent="0.3">
       <c r="I41" s="4"/>
@@ -2764,15 +2764,42 @@
     </row>
   </sheetData>
   <mergeCells count="59">
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="L15:M15"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="L16:M16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="L17:M17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="L22:M22"/>
     <mergeCell ref="F30:G30"/>
     <mergeCell ref="F23:G23"/>
     <mergeCell ref="L23:M23"/>
@@ -2787,42 +2814,15 @@
     <mergeCell ref="F27:G27"/>
     <mergeCell ref="F28:G28"/>
     <mergeCell ref="F29:G29"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="L20:M20"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="L21:M21"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="L14:M14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="L15:M15"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="L16:M16"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="F34:G34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>